<commit_message>
validacion de conflictos OC-Proveedor y manejo de errores
</commit_message>
<xml_diff>
--- a/uploads/PACKING LIST NACIONAL (PROSA-KOBBO PEG) REF.657.xlsx
+++ b/uploads/PACKING LIST NACIONAL (PROSA-KOBBO PEG) REF.657.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maverick.morales\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7BB375D-1422-483F-B377-FA957F2C67C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6AE4912-2B12-43FF-9395-B4A62C374087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2070" yWindow="735" windowWidth="15375" windowHeight="7785" activeTab="1" xr2:uid="{2B1E1A3D-0DD1-4216-B84E-CA00142C0949}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{2B1E1A3D-0DD1-4216-B84E-CA00142C0949}"/>
   </bookViews>
   <sheets>
     <sheet name="PL DETALLE" sheetId="1" r:id="rId1"/>
@@ -88,12 +88,6 @@
     <t xml:space="preserve">RPEG                </t>
   </si>
   <si>
-    <t>IMPORTADORA Y COMERCIALIZADORA PROSA CHILE SPA</t>
-  </si>
-  <si>
-    <t>PUBLICIDAD E INVERSIONES KOBBO SPA</t>
-  </si>
-  <si>
     <t>7688804500017078</t>
   </si>
   <si>
@@ -158,6 +152,12 @@
   </si>
   <si>
     <t>PROSA</t>
+  </si>
+  <si>
+    <t>PRUEBA</t>
+  </si>
+  <si>
+    <t>PRUEBA 2</t>
   </si>
 </sst>
 </file>
@@ -364,6 +364,30 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -371,30 +395,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
@@ -740,15 +740,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -775,16 +775,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>19</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>14</v>
@@ -798,16 +798,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>14</v>
@@ -821,16 +821,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>14</v>
@@ -844,16 +844,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>14</v>
@@ -867,16 +867,16 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>14</v>
@@ -890,16 +890,16 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>14</v>
@@ -913,16 +913,16 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>14</v>
@@ -936,16 +936,16 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>14</v>
@@ -959,16 +959,16 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>14</v>
@@ -982,16 +982,16 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>14</v>
@@ -1005,16 +1005,16 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>14</v>
@@ -1028,16 +1028,16 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>14</v>
@@ -1051,16 +1051,16 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>14</v>
@@ -1074,16 +1074,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>14</v>
@@ -1097,16 +1097,16 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>14</v>
@@ -1120,16 +1120,16 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>38</v>
-      </c>
       <c r="C18" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>14</v>
@@ -1152,10 +1152,10 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="13"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="21"/>
       <c r="F20" s="2">
         <f>+SUM(F3:F19)</f>
         <v>16</v>
@@ -1199,14 +1199,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
     </row>
     <row r="2" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -1239,7 +1239,7 @@
         <v>13</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="E3" s="6">
         <v>7</v>
@@ -1250,7 +1250,7 @@
     </row>
     <row r="4" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6">
-        <v>39984</v>
+        <v>39669</v>
       </c>
       <c r="B4" s="6">
         <v>9523</v>
@@ -1259,18 +1259,18 @@
         <v>13</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="E4" s="6">
         <v>9</v>
       </c>
-      <c r="F4" s="21"/>
+      <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
+      <c r="D5" s="11"/>
       <c r="E5" s="7"/>
       <c r="F5" s="6"/>
     </row>
@@ -1308,33 +1308,33 @@
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="20"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="18"/>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="20"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="18"/>
     </row>
     <row r="11" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="13">
         <v>46178</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="15"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:F6" xr:uid="{F1A63DEB-9037-485B-8B18-0D7D96E77363}">

</xml_diff>